<commit_message>
port 9mm stats, normalize velocities
</commit_message>
<xml_diff>
--- a/changes/9mm-barrels.xlsx
+++ b/changes/9mm-barrels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA2EEEEA-549A-4790-84A6-85F1ED36F1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60816E63-E791-45B7-BFF3-88F4534D7E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -714,8 +714,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -969,19 +970,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U40"/>
+  <dimension ref="A1:W40"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" customWidth="1"/>
     <col min="2" max="2" width="45.85546875" customWidth="1"/>
+    <col min="22" max="23" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1040,7 +1042,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1066,14 +1068,14 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>-61</v>
+        <v>-50</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
       <c r="N3">
         <f>C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*10+J3/300+G3/1.3</f>
-        <v>-2.2033333333333331</v>
+        <v>-2.1666666666666665</v>
       </c>
       <c r="P3">
         <v>0</v>
@@ -1089,8 +1091,16 @@
         <f>ROUND((Q3-5)*0.09/11, 2)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V3" s="1">
+        <f>(Q3-6)*35</f>
+        <v>-52.913349999999987</v>
+      </c>
+      <c r="W3" s="1">
+        <f>V3+1200</f>
+        <v>1147.08665</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>76</v>
       </c>
@@ -1121,22 +1131,38 @@
       <c r="M4">
         <v>2000</v>
       </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V4" s="1">
+        <f t="shared" ref="V4:V40" si="0">(Q4-6)*35</f>
+        <v>-210</v>
+      </c>
+      <c r="W4" s="1">
+        <f t="shared" ref="W4:W40" si="1">V4+1200</f>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="N5">
-        <f t="shared" ref="N5:N40" si="0">C5-D5*20-E5*0.8-F5*0.6-H5*7.5+I5*15+J5/300</f>
+        <f t="shared" ref="N5:N40" si="2">C5-D5*20-E5*0.8-F5*0.6-H5*7.5+I5*15+J5/300</f>
         <v>0</v>
       </c>
       <c r="S5">
-        <f t="shared" ref="S5:S40" si="1">ROUND(Q5*0.024+P5+R5,2)</f>
+        <f t="shared" ref="S5:S40" si="3">ROUND(Q5*0.024+P5+R5,2)</f>
         <v>0</v>
       </c>
       <c r="T5">
-        <f t="shared" ref="T5:T40" si="2">ROUND((Q5-5)*0.09/11, 2)</f>
+        <f t="shared" ref="T5:T40" si="4">ROUND((Q5-5)*0.09/11, 2)</f>
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V5" s="1">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+      <c r="W5" s="1">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -1162,14 +1188,14 @@
         <v>-0.02</v>
       </c>
       <c r="J6">
-        <v>-80</v>
+        <v>-70</v>
       </c>
       <c r="M6">
         <v>1000</v>
       </c>
       <c r="N6">
-        <f t="shared" si="0"/>
-        <v>-3.3166666666666664</v>
+        <f t="shared" si="2"/>
+        <v>-3.2833333333333332</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -1178,15 +1204,23 @@
         <v>3.9</v>
       </c>
       <c r="S6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.09</v>
       </c>
       <c r="T6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.01</v>
       </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V6" s="1">
+        <f t="shared" si="0"/>
+        <v>-73.5</v>
+      </c>
+      <c r="W6" s="1">
+        <f t="shared" si="1"/>
+        <v>1126.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1218,7 +1252,7 @@
         <v>3000</v>
       </c>
       <c r="N7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-3.1416666666666666</v>
       </c>
       <c r="P7">
@@ -1228,15 +1262,23 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="S7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.11</v>
       </c>
       <c r="T7">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V7" s="1">
+        <f t="shared" si="0"/>
+        <v>-49.000000000000014</v>
+      </c>
+      <c r="W7" s="1">
+        <f t="shared" si="1"/>
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1262,14 +1304,14 @@
         <v>0</v>
       </c>
       <c r="J8">
-        <v>-45</v>
+        <v>-46</v>
       </c>
       <c r="M8">
         <v>0</v>
       </c>
       <c r="N8">
-        <f t="shared" si="0"/>
-        <v>-2.35</v>
+        <f t="shared" si="2"/>
+        <v>-2.3533333333333335</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1278,15 +1320,23 @@
         <v>4.7</v>
       </c>
       <c r="S8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.11</v>
       </c>
       <c r="T8">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V8" s="1">
+        <f t="shared" si="0"/>
+        <v>-45.499999999999993</v>
+      </c>
+      <c r="W8" s="1">
+        <f t="shared" si="1"/>
+        <v>1154.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -1312,14 +1362,14 @@
         <v>0.02</v>
       </c>
       <c r="J9">
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="M9">
         <v>1500</v>
       </c>
       <c r="N9">
-        <f t="shared" ref="N9:N16" si="3">C9-D9*20-E9*0.8-F9*0.6-H9*5+I9*10+J9/300+G9/1.3</f>
-        <v>-3.5333333333333332</v>
+        <f t="shared" ref="N9:N16" si="5">C9-D9*20-E9*0.8-F9*0.6-H9*5+I9*10+J9/300+G9/1.3</f>
+        <v>-3.5666666666666669</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -1328,29 +1378,45 @@
         <v>5.5</v>
       </c>
       <c r="S9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.13</v>
       </c>
       <c r="T9">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V9" s="1">
+        <f t="shared" si="0"/>
+        <v>-17.5</v>
+      </c>
+      <c r="W9" s="1">
+        <f t="shared" si="1"/>
+        <v>1182.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="N10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="S10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V10" s="1">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+      <c r="W10" s="1">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -1376,14 +1442,14 @@
         <v>0</v>
       </c>
       <c r="J11">
-        <v>-78</v>
+        <v>-70</v>
       </c>
       <c r="M11">
         <v>0</v>
       </c>
       <c r="N11">
-        <f t="shared" si="3"/>
-        <v>-2.2599999999999998</v>
+        <f t="shared" si="5"/>
+        <v>-2.2333333333333334</v>
       </c>
       <c r="P11">
         <v>0</v>
@@ -1392,15 +1458,23 @@
         <v>4.0157499999999997</v>
       </c>
       <c r="S11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.1</v>
       </c>
       <c r="T11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.01</v>
       </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V11" s="1">
+        <f t="shared" si="0"/>
+        <v>-69.448750000000004</v>
+      </c>
+      <c r="W11" s="1">
+        <f t="shared" si="1"/>
+        <v>1130.55125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -1426,14 +1500,14 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>-44</v>
+        <v>-40</v>
       </c>
       <c r="M12">
         <v>750</v>
       </c>
       <c r="N12">
-        <f t="shared" si="3"/>
-        <v>-6.8466666666666667</v>
+        <f t="shared" si="5"/>
+        <v>-6.8333333333333339</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -1442,29 +1516,45 @@
         <v>5</v>
       </c>
       <c r="S12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.12</v>
       </c>
       <c r="T12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V12" s="1">
+        <f t="shared" si="0"/>
+        <v>-35</v>
+      </c>
+      <c r="W12" s="1">
+        <f t="shared" si="1"/>
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="N13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="S13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V13" s="1">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+      <c r="W13" s="1">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>34</v>
       </c>
@@ -1490,14 +1580,14 @@
         <v>0.03</v>
       </c>
       <c r="J14">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="M14">
         <v>0</v>
       </c>
       <c r="N14">
-        <f t="shared" si="3"/>
-        <v>0.85666666666666713</v>
+        <f t="shared" si="5"/>
+        <v>1.0333333333333337</v>
       </c>
       <c r="P14">
         <v>0.04</v>
@@ -1506,15 +1596,23 @@
         <v>8.8582699999999992</v>
       </c>
       <c r="S14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.25</v>
       </c>
       <c r="T14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.03</v>
       </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V14" s="1">
+        <f t="shared" si="0"/>
+        <v>100.03944999999997</v>
+      </c>
+      <c r="W14" s="1">
+        <f t="shared" si="1"/>
+        <v>1300.03945</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -1546,7 +1644,7 @@
         <v>1000</v>
       </c>
       <c r="N15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.81666666666666621</v>
       </c>
       <c r="P15">
@@ -1556,29 +1654,45 @@
         <v>5.74803</v>
       </c>
       <c r="S15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.18</v>
       </c>
       <c r="T15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.01</v>
       </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V15" s="1">
+        <f t="shared" si="0"/>
+        <v>-8.818950000000001</v>
+      </c>
+      <c r="W15" s="1">
+        <f t="shared" si="1"/>
+        <v>1191.1810499999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="N16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="S16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V16" s="1">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+      <c r="W16" s="1">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>38</v>
       </c>
@@ -1604,14 +1718,14 @@
         <v>-0.03</v>
       </c>
       <c r="J17">
-        <v>-300</v>
+        <v>-100</v>
       </c>
       <c r="M17">
         <v>750</v>
       </c>
       <c r="N17">
-        <f t="shared" si="0"/>
-        <v>-8.3250000000000011</v>
+        <f t="shared" si="2"/>
+        <v>-7.6583333333333341</v>
       </c>
       <c r="P17">
         <v>0.04</v>
@@ -1620,15 +1734,23 @@
         <v>3</v>
       </c>
       <c r="S17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.11</v>
       </c>
       <c r="T17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.02</v>
       </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V17" s="1">
+        <f t="shared" si="0"/>
+        <v>-105</v>
+      </c>
+      <c r="W17" s="1">
+        <f t="shared" si="1"/>
+        <v>1095</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -1654,14 +1776,14 @@
         <v>0</v>
       </c>
       <c r="J18">
-        <v>-225</v>
+        <v>-40</v>
       </c>
       <c r="M18">
         <v>800</v>
       </c>
       <c r="N18">
-        <f t="shared" si="0"/>
-        <v>-7.65</v>
+        <f t="shared" si="2"/>
+        <v>-7.0333333333333341</v>
       </c>
       <c r="P18">
         <v>0.04</v>
@@ -1670,15 +1792,23 @@
         <v>5</v>
       </c>
       <c r="S18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.16</v>
       </c>
       <c r="T18">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V18" s="1">
+        <f t="shared" si="0"/>
+        <v>-35</v>
+      </c>
+      <c r="W18" s="1">
+        <f t="shared" si="1"/>
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -1704,14 +1834,14 @@
         <v>0.03</v>
       </c>
       <c r="J19">
-        <v>-90</v>
+        <v>90</v>
       </c>
       <c r="M19">
         <v>900</v>
       </c>
       <c r="N19">
-        <f t="shared" si="0"/>
-        <v>-6.9750000000000005</v>
+        <f t="shared" si="2"/>
+        <v>-6.3750000000000009</v>
       </c>
       <c r="P19">
         <v>0.04</v>
@@ -1720,15 +1850,23 @@
         <v>8.5</v>
       </c>
       <c r="S19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.24</v>
       </c>
       <c r="T19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.03</v>
       </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V19" s="1">
+        <f t="shared" si="0"/>
+        <v>87.5</v>
+      </c>
+      <c r="W19" s="1">
+        <f t="shared" si="1"/>
+        <v>1287.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -1754,14 +1892,14 @@
         <v>0.04</v>
       </c>
       <c r="J20">
-        <v>-70</v>
+        <v>110</v>
       </c>
       <c r="M20">
         <v>950</v>
       </c>
       <c r="N20">
-        <f t="shared" si="0"/>
-        <v>-7.0083333333333346</v>
+        <f t="shared" si="2"/>
+        <v>-6.408333333333335</v>
       </c>
       <c r="P20">
         <v>0.04</v>
@@ -1770,15 +1908,23 @@
         <v>9</v>
       </c>
       <c r="S20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.26</v>
       </c>
       <c r="T20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.03</v>
       </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V20" s="1">
+        <f t="shared" si="0"/>
+        <v>105</v>
+      </c>
+      <c r="W20" s="1">
+        <f t="shared" si="1"/>
+        <v>1305</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -1810,7 +1956,7 @@
         <v>0</v>
       </c>
       <c r="N21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-8.3833333333333346</v>
       </c>
       <c r="P21">
@@ -1820,15 +1966,23 @@
         <v>16</v>
       </c>
       <c r="S21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.42</v>
       </c>
       <c r="T21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.09</v>
       </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V21" s="1">
+        <f t="shared" si="0"/>
+        <v>350</v>
+      </c>
+      <c r="W21" s="1">
+        <f t="shared" si="1"/>
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>48</v>
       </c>
@@ -1860,7 +2014,7 @@
         <v>1200</v>
       </c>
       <c r="N22">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-8.1833333333333336</v>
       </c>
       <c r="P22">
@@ -1873,15 +2027,23 @@
         <v>0.01</v>
       </c>
       <c r="S22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.43</v>
       </c>
       <c r="T22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.09</v>
       </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V22" s="1">
+        <f t="shared" si="0"/>
+        <v>350</v>
+      </c>
+      <c r="W22" s="1">
+        <f t="shared" si="1"/>
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>50</v>
       </c>
@@ -1913,7 +2075,7 @@
         <v>1200</v>
       </c>
       <c r="N23">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-7.9833333333333352</v>
       </c>
       <c r="P23">
@@ -1926,29 +2088,45 @@
         <v>0.02</v>
       </c>
       <c r="S23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.44</v>
       </c>
       <c r="T23">
+        <f t="shared" si="4"/>
+        <v>0.09</v>
+      </c>
+      <c r="V23" s="1">
+        <f t="shared" si="0"/>
+        <v>350</v>
+      </c>
+      <c r="W23" s="1">
+        <f t="shared" si="1"/>
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="N24">
         <f t="shared" si="2"/>
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="N24">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T24">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V24" s="1">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+      <c r="W24" s="1">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>52</v>
       </c>
@@ -1974,14 +2152,14 @@
         <v>0.04</v>
       </c>
       <c r="J25">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="M25">
         <v>0</v>
       </c>
       <c r="N25">
-        <f t="shared" si="0"/>
-        <v>-6.0083333333333337</v>
+        <f t="shared" si="2"/>
+        <v>-5.7750000000000004</v>
       </c>
       <c r="P25">
         <v>0.04</v>
@@ -1990,15 +2168,23 @@
         <v>9.3700799999999997</v>
       </c>
       <c r="S25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.26</v>
       </c>
       <c r="T25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.04</v>
       </c>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V25" s="1">
+        <f t="shared" si="0"/>
+        <v>117.9528</v>
+      </c>
+      <c r="W25" s="1">
+        <f t="shared" si="1"/>
+        <v>1317.9528</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>54</v>
       </c>
@@ -2024,14 +2210,14 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="J26">
-        <v>90</v>
+        <v>170</v>
       </c>
       <c r="M26">
         <v>500</v>
       </c>
       <c r="N26">
-        <f t="shared" si="0"/>
-        <v>-6.6500000000000021</v>
+        <f t="shared" si="2"/>
+        <v>-6.3833333333333355</v>
       </c>
       <c r="P26">
         <v>0.04</v>
@@ -2040,29 +2226,45 @@
         <v>13.582700000000001</v>
       </c>
       <c r="S26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.37</v>
       </c>
       <c r="T26">
+        <f t="shared" si="4"/>
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="V26" s="1">
+        <f t="shared" si="0"/>
+        <v>265.39450000000005</v>
+      </c>
+      <c r="W26" s="1">
+        <f t="shared" si="1"/>
+        <v>1465.3945000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="N27">
         <f t="shared" si="2"/>
-        <v>7.0000000000000007E-2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="N27">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T27">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V27" s="1">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+      <c r="W27" s="1">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>56</v>
       </c>
@@ -2088,14 +2290,14 @@
         <v>0.09</v>
       </c>
       <c r="J28">
-        <v>145</v>
+        <v>200</v>
       </c>
       <c r="M28">
         <v>2000</v>
       </c>
       <c r="N28">
-        <f t="shared" si="0"/>
-        <v>12.433333333333334</v>
+        <f t="shared" si="2"/>
+        <v>12.616666666666667</v>
       </c>
       <c r="P28">
         <v>0.04</v>
@@ -2104,15 +2306,23 @@
         <v>16.535399999999999</v>
       </c>
       <c r="S28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.44</v>
       </c>
       <c r="T28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.09</v>
       </c>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V28" s="1">
+        <f t="shared" si="0"/>
+        <v>368.73899999999998</v>
+      </c>
+      <c r="W28" s="1">
+        <f t="shared" si="1"/>
+        <v>1568.739</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>58</v>
       </c>
@@ -2138,14 +2348,14 @@
         <v>0.06</v>
       </c>
       <c r="J29">
-        <v>105</v>
+        <v>160</v>
       </c>
       <c r="M29">
         <v>3000</v>
       </c>
       <c r="N29">
-        <f t="shared" si="0"/>
-        <v>8.1</v>
+        <f t="shared" si="2"/>
+        <v>8.2833333333333332</v>
       </c>
       <c r="P29">
         <v>0.04</v>
@@ -2154,29 +2364,45 @@
         <v>12.795299999999999</v>
       </c>
       <c r="S29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.35</v>
       </c>
       <c r="T29">
+        <f t="shared" si="4"/>
+        <v>0.06</v>
+      </c>
+      <c r="V29" s="1">
+        <f t="shared" si="0"/>
+        <v>237.83549999999997</v>
+      </c>
+      <c r="W29" s="1">
+        <f t="shared" si="1"/>
+        <v>1437.8354999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="N30">
         <f t="shared" si="2"/>
-        <v>0.06</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="N30">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S30">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V30" s="1">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+      <c r="W30" s="1">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>60</v>
       </c>
@@ -2199,14 +2425,14 @@
         <v>0</v>
       </c>
       <c r="J31">
-        <v>-15</v>
+        <v>70</v>
       </c>
       <c r="M31">
         <v>500</v>
       </c>
       <c r="N31">
-        <f t="shared" si="0"/>
-        <v>-4.8500000000000005</v>
+        <f t="shared" si="2"/>
+        <v>-4.5666666666666673</v>
       </c>
       <c r="P31">
         <v>0.04</v>
@@ -2215,15 +2441,23 @@
         <v>8</v>
       </c>
       <c r="S31">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.23</v>
       </c>
       <c r="T31">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.02</v>
       </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V31" s="1">
+        <f t="shared" si="0"/>
+        <v>70</v>
+      </c>
+      <c r="W31" s="1">
+        <f t="shared" si="1"/>
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -2246,14 +2480,14 @@
         <v>0.05</v>
       </c>
       <c r="J32">
-        <v>-20</v>
+        <v>70</v>
       </c>
       <c r="M32">
         <v>1000</v>
       </c>
       <c r="N32">
-        <f t="shared" si="0"/>
-        <v>-9.4416666666666664</v>
+        <f t="shared" si="2"/>
+        <v>-9.1416666666666675</v>
       </c>
       <c r="P32">
         <v>0.04</v>
@@ -2262,29 +2496,45 @@
         <v>8</v>
       </c>
       <c r="S32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.23</v>
       </c>
       <c r="T32">
+        <f t="shared" si="4"/>
+        <v>0.02</v>
+      </c>
+      <c r="V32" s="1">
+        <f t="shared" si="0"/>
+        <v>70</v>
+      </c>
+      <c r="W32" s="1">
+        <f t="shared" si="1"/>
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="N33">
         <f t="shared" si="2"/>
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="N33">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S33">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T33">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V33" s="1">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+      <c r="W33" s="1">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>64</v>
       </c>
@@ -2310,7 +2560,7 @@
         <v>0</v>
       </c>
       <c r="J34">
-        <v>-28</v>
+        <v>-20</v>
       </c>
       <c r="K34">
         <v>0</v>
@@ -2319,8 +2569,8 @@
         <v>800</v>
       </c>
       <c r="N34">
-        <f t="shared" si="0"/>
-        <v>-4.6933333333333342</v>
+        <f t="shared" si="2"/>
+        <v>-4.666666666666667</v>
       </c>
       <c r="P34">
         <v>0.04</v>
@@ -2329,15 +2579,23 @@
         <v>5.5118099999999997</v>
       </c>
       <c r="S34">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.17</v>
       </c>
       <c r="T34">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V34" s="1">
+        <f t="shared" si="0"/>
+        <v>-17.086650000000013</v>
+      </c>
+      <c r="W34" s="1">
+        <f t="shared" si="1"/>
+        <v>1182.91335</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>66</v>
       </c>
@@ -2363,7 +2621,7 @@
         <v>0.02</v>
       </c>
       <c r="J35">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="K35">
         <v>-0.1</v>
@@ -2372,8 +2630,8 @@
         <v>750</v>
       </c>
       <c r="N35">
-        <f t="shared" si="0"/>
-        <v>-4.1183333333333341</v>
+        <f t="shared" si="2"/>
+        <v>-4.0583333333333345</v>
       </c>
       <c r="P35">
         <v>0.04</v>
@@ -2382,29 +2640,45 @@
         <v>6.6929100000000004</v>
       </c>
       <c r="S35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.2</v>
       </c>
       <c r="T35">
+        <f t="shared" si="4"/>
+        <v>0.01</v>
+      </c>
+      <c r="V35" s="1">
+        <f t="shared" si="0"/>
+        <v>24.251850000000012</v>
+      </c>
+      <c r="W35" s="1">
+        <f t="shared" si="1"/>
+        <v>1224.2518500000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="N36">
         <f t="shared" si="2"/>
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="N36">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V36" s="1">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+      <c r="W36" s="1">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>68</v>
       </c>
@@ -2436,22 +2710,30 @@
         <v>1500</v>
       </c>
       <c r="N37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11.66</v>
       </c>
       <c r="P37">
         <v>0.03</v>
       </c>
       <c r="S37">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.03</v>
       </c>
       <c r="T37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.04</v>
       </c>
-    </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V37" s="1">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+      <c r="W37" s="1">
+        <f t="shared" si="1"/>
+        <v>990</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>70</v>
       </c>
@@ -2483,7 +2765,7 @@
         <v>1200</v>
       </c>
       <c r="N38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>8.4350000000000005</v>
       </c>
       <c r="P38">
@@ -2493,15 +2775,23 @@
         <v>4.5</v>
       </c>
       <c r="S38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.14000000000000001</v>
       </c>
       <c r="T38">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V38" s="1">
+        <f t="shared" si="0"/>
+        <v>-52.5</v>
+      </c>
+      <c r="W38" s="1">
+        <f t="shared" si="1"/>
+        <v>1147.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>72</v>
       </c>
@@ -2533,7 +2823,7 @@
         <v>1500</v>
       </c>
       <c r="N39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>15.353333333333333</v>
       </c>
       <c r="P39">
@@ -2543,15 +2833,23 @@
         <v>6.0236200000000002</v>
       </c>
       <c r="S39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.17</v>
       </c>
       <c r="T39">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.01</v>
       </c>
-    </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="V39" s="1">
+        <f t="shared" si="0"/>
+        <v>0.82670000000000687</v>
+      </c>
+      <c r="W39" s="1">
+        <f t="shared" si="1"/>
+        <v>1200.8267000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>74</v>
       </c>
@@ -2583,7 +2881,7 @@
         <v>3000</v>
       </c>
       <c r="N40">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-12.683333333333334</v>
       </c>
       <c r="P40">
@@ -2593,12 +2891,20 @@
         <v>15.984252</v>
       </c>
       <c r="S40">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.41</v>
       </c>
       <c r="T40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.09</v>
+      </c>
+      <c r="V40" s="1">
+        <f t="shared" si="0"/>
+        <v>349.44882000000001</v>
+      </c>
+      <c r="W40" s="1">
+        <f t="shared" si="1"/>
+        <v>1549.4488200000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>